<commit_message>
add nos dependency 279bb61b7f9d11b1844a23a2bc4a64f1f2eed9a7
</commit_message>
<xml_diff>
--- a/ig/nr-update-location-identifier/ValueSet-fr-core-civility.xlsx
+++ b/ig/nr-update-location-identifier/ValueSet-fr-core-civility.xlsx
@@ -7,7 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Metadata" r:id="rId3" sheetId="1"/>
-    <sheet name="Include from TRE-R81-Civilite" r:id="rId4" sheetId="2"/>
+    <sheet name="Include from TRE_R81-Civilite" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-12-20T15:16:44+00:00</t>
+    <t>2023-12-20T16:57:20+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>